<commit_message>
added multiple teachers for excel export and import at path api/importExcel/{filename} to import
</commit_message>
<xml_diff>
--- a/leo-planer/src/files/excelFiles/export/test1.xlsx
+++ b/leo-planer/src/files/excelFiles/export/test1.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="153">
   <si>
     <t>CSI Id</t>
   </si>
@@ -48,13 +48,7 @@
     <t>Subject Id</t>
   </si>
   <si>
-    <t>Subject Symbol</t>
-  </si>
-  <si>
-    <t>Teacher Id</t>
-  </si>
-  <si>
-    <t>Teacher Symbol</t>
+    <t>Teacher Ids</t>
   </si>
   <si>
     <t>Weekly Hours</t>
@@ -66,423 +60,414 @@
     <t>Is better as Double Period</t>
   </si>
   <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Symbol</t>
+  </si>
+  <si>
+    <t>Required Room Types</t>
+  </si>
+  <si>
+    <t>angewandte mathematik</t>
+  </si>
+  <si>
+    <t>am</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>naturwissenschaften physik</t>
+  </si>
+  <si>
+    <t>nwp</t>
+  </si>
+  <si>
+    <t>PHY</t>
+  </si>
+  <si>
+    <t>geschichte</t>
+  </si>
+  <si>
+    <t>ges</t>
+  </si>
+  <si>
+    <t>biologie</t>
+  </si>
+  <si>
+    <t>bio</t>
+  </si>
+  <si>
+    <t>naturwissenschaften chemie</t>
+  </si>
+  <si>
+    <t>nwc</t>
+  </si>
+  <si>
+    <t>CHEM, PHY</t>
+  </si>
+  <si>
+    <t>recht</t>
+  </si>
+  <si>
+    <t>wirtschaft</t>
+  </si>
+  <si>
+    <t>wt</t>
+  </si>
+  <si>
+    <t>englisch</t>
+  </si>
+  <si>
     <t>eng</t>
   </si>
   <si>
+    <t>geographie</t>
+  </si>
+  <si>
+    <t>geo</t>
+  </si>
+  <si>
+    <t>software entwicklung</t>
+  </si>
+  <si>
+    <t>sew</t>
+  </si>
+  <si>
+    <t>deutsch</t>
+  </si>
+  <si>
+    <t>de</t>
+  </si>
+  <si>
+    <t>informationssysteme</t>
+  </si>
+  <si>
+    <t>insy</t>
+  </si>
+  <si>
+    <t>informationstechnische projekte</t>
+  </si>
+  <si>
+    <t>itp</t>
+  </si>
+  <si>
+    <t>religion</t>
+  </si>
+  <si>
+    <t>rel</t>
+  </si>
+  <si>
+    <t>medientechnik print und design</t>
+  </si>
+  <si>
+    <t>medtpd</t>
+  </si>
+  <si>
+    <t>medientechnik mobile computing</t>
+  </si>
+  <si>
+    <t>medtmc</t>
+  </si>
+  <si>
+    <t>medientechnik film und audio</t>
+  </si>
+  <si>
+    <t>medtfi</t>
+  </si>
+  <si>
+    <t>medientechnik social media</t>
+  </si>
+  <si>
+    <t>medtsm</t>
+  </si>
+  <si>
+    <t>medientechnik virtuelle welten und spieleentwicklung</t>
+  </si>
+  <si>
+    <t>medt3d</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>Short</t>
+  </si>
+  <si>
+    <t>Room Type</t>
+  </si>
+  <si>
+    <t>potts</t>
+  </si>
+  <si>
+    <t>pot</t>
+  </si>
+  <si>
+    <t>WORKSHOP</t>
+  </si>
+  <si>
+    <t>vincent</t>
+  </si>
+  <si>
+    <t>vin</t>
+  </si>
+  <si>
+    <t>williams</t>
+  </si>
+  <si>
+    <t>wil</t>
+  </si>
+  <si>
+    <t>morgan</t>
+  </si>
+  <si>
+    <t>mor</t>
+  </si>
+  <si>
+    <t>WORKSHOP, CLASSROOM</t>
+  </si>
+  <si>
+    <t>hernandez</t>
+  </si>
+  <si>
+    <t>her</t>
+  </si>
+  <si>
+    <t>SPORT, EDV</t>
+  </si>
+  <si>
+    <t>CLASSROOM, WORKSHOP</t>
+  </si>
+  <si>
+    <t>cervantes</t>
+  </si>
+  <si>
+    <t>cer</t>
+  </si>
+  <si>
+    <t>SPORT</t>
+  </si>
+  <si>
+    <t>mercado</t>
+  </si>
+  <si>
+    <t>mer</t>
+  </si>
+  <si>
+    <t>SPORT, WORKSHOP</t>
+  </si>
+  <si>
+    <t>stanton</t>
+  </si>
+  <si>
+    <t>sta</t>
+  </si>
+  <si>
+    <t>russell</t>
+  </si>
+  <si>
+    <t>rus</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t>Teaching Subjects Ids</t>
+  </si>
+  <si>
+    <t>Jill Patterson</t>
+  </si>
+  <si>
+    <t>JP</t>
+  </si>
+  <si>
+    <t>Christopher Cochran</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>16, 19, 8</t>
+  </si>
+  <si>
+    <t>Shane Allen</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Austin Burton</t>
+  </si>
+  <si>
+    <t>AB</t>
+  </si>
+  <si>
+    <t>19, 14, 9</t>
+  </si>
+  <si>
+    <t>Sean Burnett</t>
+  </si>
+  <si>
+    <t>SB</t>
+  </si>
+  <si>
+    <t>Abigail Sullivan</t>
+  </si>
+  <si>
+    <t>AS</t>
+  </si>
+  <si>
+    <t>8, 2</t>
+  </si>
+  <si>
+    <t>Teresa Baker</t>
+  </si>
+  <si>
+    <t>TB</t>
+  </si>
+  <si>
+    <t>2, 17</t>
+  </si>
+  <si>
+    <t>James Wood</t>
+  </si>
+  <si>
+    <t>JW</t>
+  </si>
+  <si>
+    <t>Monique Ware</t>
+  </si>
+  <si>
+    <t>MW</t>
+  </si>
+  <si>
+    <t>19, 15, 7</t>
+  </si>
+  <si>
+    <t>Sarah Rivera</t>
+  </si>
+  <si>
+    <t>SR</t>
+  </si>
+  <si>
+    <t>2, 13, 14</t>
+  </si>
+  <si>
+    <t>Samantha Larson</t>
+  </si>
+  <si>
     <t>SL</t>
   </si>
   <si>
-    <t>insy</t>
-  </si>
-  <si>
-    <t>SA</t>
-  </si>
-  <si>
-    <t>am</t>
-  </si>
-  <si>
-    <t>AS</t>
-  </si>
-  <si>
-    <t>recht</t>
-  </si>
-  <si>
-    <t>SB</t>
-  </si>
-  <si>
-    <t>medtfi</t>
-  </si>
-  <si>
-    <t>JW</t>
-  </si>
-  <si>
-    <t>geo</t>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Scott Duffy</t>
+  </si>
+  <si>
+    <t>SD</t>
+  </si>
+  <si>
+    <t>Andrew Jackson</t>
+  </si>
+  <si>
+    <t>AJ</t>
+  </si>
+  <si>
+    <t>Michael Mckinney</t>
+  </si>
+  <si>
+    <t>MM</t>
+  </si>
+  <si>
+    <t>19, 4, 5</t>
+  </si>
+  <si>
+    <t>Brian Wood</t>
+  </si>
+  <si>
+    <t>BW</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Steven Martinez</t>
   </si>
   <si>
     <t>SM</t>
   </si>
   <si>
-    <t>CC</t>
+    <t>5, 1</t>
+  </si>
+  <si>
+    <t>Jordan Fletcher</t>
   </si>
   <si>
     <t>JF</t>
   </si>
   <si>
-    <t>MW</t>
-  </si>
-  <si>
-    <t>medt3d</t>
+    <t>14, 15, 9</t>
+  </si>
+  <si>
+    <t>Riley Gutierrez</t>
+  </si>
+  <si>
+    <t>RG</t>
+  </si>
+  <si>
+    <t>4, 8, 3</t>
+  </si>
+  <si>
+    <t>Nathan King</t>
   </si>
   <si>
     <t>NK</t>
   </si>
   <si>
-    <t>sew</t>
-  </si>
-  <si>
-    <t>BW</t>
-  </si>
-  <si>
-    <t>nwc</t>
-  </si>
-  <si>
-    <t>SD</t>
-  </si>
-  <si>
-    <t>ges</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Symbol</t>
-  </si>
-  <si>
-    <t>Required Room Types</t>
-  </si>
-  <si>
-    <t>angewandte mathematik</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>naturwissenschaften physik</t>
-  </si>
-  <si>
-    <t>nwp</t>
-  </si>
-  <si>
-    <t>PHY</t>
-  </si>
-  <si>
-    <t>geschichte</t>
-  </si>
-  <si>
-    <t>biologie</t>
-  </si>
-  <si>
-    <t>bio</t>
-  </si>
-  <si>
-    <t>naturwissenschaften chemie</t>
-  </si>
-  <si>
-    <t>CHEM, PHY</t>
-  </si>
-  <si>
-    <t>wirtschaft</t>
-  </si>
-  <si>
-    <t>wt</t>
-  </si>
-  <si>
-    <t>englisch</t>
-  </si>
-  <si>
-    <t>geographie</t>
-  </si>
-  <si>
-    <t>software entwicklung</t>
-  </si>
-  <si>
-    <t>deutsch</t>
-  </si>
-  <si>
-    <t>de</t>
-  </si>
-  <si>
-    <t>informationssysteme</t>
-  </si>
-  <si>
-    <t>informationstechnische projekte</t>
-  </si>
-  <si>
-    <t>itp</t>
-  </si>
-  <si>
-    <t>religion</t>
-  </si>
-  <si>
-    <t>rel</t>
-  </si>
-  <si>
-    <t>medientechnik print und design</t>
-  </si>
-  <si>
-    <t>medtpd</t>
-  </si>
-  <si>
-    <t>medientechnik mobile computing</t>
-  </si>
-  <si>
-    <t>medtmc</t>
-  </si>
-  <si>
-    <t>medientechnik film und audio</t>
-  </si>
-  <si>
-    <t>medientechnik social media</t>
-  </si>
-  <si>
-    <t>medtsm</t>
-  </si>
-  <si>
-    <t>medientechnik virtuelle welten und spieleentwicklung</t>
-  </si>
-  <si>
-    <t>Number</t>
-  </si>
-  <si>
-    <t>Short</t>
-  </si>
-  <si>
-    <t>Room Type</t>
-  </si>
-  <si>
-    <t>potts</t>
-  </si>
-  <si>
-    <t>pot</t>
-  </si>
-  <si>
-    <t>WORKSHOP</t>
-  </si>
-  <si>
-    <t>vincent</t>
-  </si>
-  <si>
-    <t>vin</t>
-  </si>
-  <si>
-    <t>williams</t>
-  </si>
-  <si>
-    <t>wil</t>
-  </si>
-  <si>
-    <t>morgan</t>
-  </si>
-  <si>
-    <t>mor</t>
-  </si>
-  <si>
-    <t>WORKSHOP, CLASSROOM</t>
-  </si>
-  <si>
-    <t>hernandez</t>
-  </si>
-  <si>
-    <t>her</t>
-  </si>
-  <si>
-    <t>SPORT, EDV</t>
-  </si>
-  <si>
-    <t>CLASSROOM, WORKSHOP</t>
-  </si>
-  <si>
-    <t>cervantes</t>
-  </si>
-  <si>
-    <t>cer</t>
-  </si>
-  <si>
-    <t>SPORT</t>
-  </si>
-  <si>
-    <t>mercado</t>
-  </si>
-  <si>
-    <t>mer</t>
-  </si>
-  <si>
-    <t>SPORT, WORKSHOP</t>
-  </si>
-  <si>
-    <t>stanton</t>
-  </si>
-  <si>
-    <t>sta</t>
-  </si>
-  <si>
-    <t>russell</t>
-  </si>
-  <si>
-    <t>rus</t>
-  </si>
-  <si>
-    <t>Id</t>
-  </si>
-  <si>
-    <t>Teaching Subjects Ids</t>
-  </si>
-  <si>
-    <t>Teaching Subjects Symbols</t>
-  </si>
-  <si>
-    <t>Jill Patterson</t>
-  </si>
-  <si>
-    <t>JP</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>Christopher Cochran</t>
-  </si>
-  <si>
-    <t>16, 19, 8</t>
-  </si>
-  <si>
-    <t>medtmc, medt3d, eng</t>
-  </si>
-  <si>
-    <t>Shane Allen</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>Austin Burton</t>
-  </si>
-  <si>
-    <t>AB</t>
-  </si>
-  <si>
-    <t>19, 14, 9</t>
-  </si>
-  <si>
-    <t>medt3d, rel, geo</t>
-  </si>
-  <si>
-    <t>Sean Burnett</t>
-  </si>
-  <si>
-    <t>Abigail Sullivan</t>
-  </si>
-  <si>
-    <t>8, 2</t>
-  </si>
-  <si>
-    <t>eng, nwp</t>
-  </si>
-  <si>
-    <t>Teresa Baker</t>
-  </si>
-  <si>
-    <t>TB</t>
-  </si>
-  <si>
-    <t>2, 17</t>
-  </si>
-  <si>
-    <t>nwp, medtfi</t>
-  </si>
-  <si>
-    <t>James Wood</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>Monique Ware</t>
-  </si>
-  <si>
-    <t>19, 15, 7</t>
-  </si>
-  <si>
-    <t>medt3d, medtpd, wt</t>
-  </si>
-  <si>
-    <t>Sarah Rivera</t>
-  </si>
-  <si>
-    <t>SR</t>
-  </si>
-  <si>
-    <t>2, 13, 14</t>
-  </si>
-  <si>
-    <t>nwp, itp, rel</t>
-  </si>
-  <si>
-    <t>Samantha Larson</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Scott Duffy</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>Andrew Jackson</t>
-  </si>
-  <si>
-    <t>AJ</t>
-  </si>
-  <si>
-    <t>Michael Mckinney</t>
-  </si>
-  <si>
-    <t>MM</t>
-  </si>
-  <si>
-    <t>19, 4, 5</t>
-  </si>
-  <si>
-    <t>medt3d, bio, nwc</t>
-  </si>
-  <si>
-    <t>Brian Wood</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Steven Martinez</t>
-  </si>
-  <si>
-    <t>5, 1</t>
-  </si>
-  <si>
-    <t>nwc, am</t>
-  </si>
-  <si>
-    <t>Jordan Fletcher</t>
-  </si>
-  <si>
-    <t>14, 15, 9</t>
-  </si>
-  <si>
-    <t>rel, medtpd, geo</t>
-  </si>
-  <si>
-    <t>Riley Gutierrez</t>
-  </si>
-  <si>
-    <t>RG</t>
-  </si>
-  <si>
-    <t>4, 8, 3</t>
-  </si>
-  <si>
-    <t>bio, eng, ges</t>
-  </si>
-  <si>
-    <t>Nathan King</t>
-  </si>
-  <si>
     <t>5, 17</t>
   </si>
   <si>
-    <t>nwc, medtfi</t>
-  </si>
-  <si>
     <t>Jake Kelley</t>
   </si>
   <si>
@@ -490,9 +475,6 @@
   </si>
   <si>
     <t>13, 3, 17</t>
-  </si>
-  <si>
-    <t>itp, ges, medtfi</t>
   </si>
 </sst>
 </file>
@@ -537,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -601,7 +583,7 @@
         <v>3.0</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="6">
@@ -689,7 +671,7 @@
         <v>14.0</v>
       </c>
       <c r="B16" t="n" s="0">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="17">
@@ -705,7 +687,7 @@
         <v>16.0</v>
       </c>
       <c r="B18" t="n" s="0">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="19">
@@ -721,7 +703,7 @@
         <v>18.0</v>
       </c>
       <c r="B20" t="n" s="0">
-        <v>13.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="21">
@@ -729,7 +711,7 @@
         <v>19.0</v>
       </c>
       <c r="B21" t="n" s="0">
-        <v>14.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="22">
@@ -737,6 +719,22 @@
         <v>20.0</v>
       </c>
       <c r="B22" t="n" s="0">
+        <v>13.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n" s="0">
+        <v>21.0</v>
+      </c>
+      <c r="B23" t="n" s="0">
+        <v>14.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n" s="0">
+        <v>22.0</v>
+      </c>
+      <c r="B24" t="n" s="0">
         <v>14.0</v>
       </c>
     </row>
@@ -747,7 +745,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -769,12 +767,6 @@
       <c r="F1" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="G1" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="H1" t="s" s="0">
-        <v>15</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
@@ -784,21 +776,15 @@
         <v>8.0</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D2" t="n" s="0">
-        <v>11.0</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="F2" t="n" s="0">
+        <v>14</v>
+      </c>
+      <c r="D2" t="n">
         <v>2.0</v>
       </c>
-      <c r="G2" t="b" s="0">
+      <c r="E2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" t="b" s="0">
+      <c r="F2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -810,21 +796,15 @@
         <v>12.0</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="D3" t="n" s="0">
-        <v>3.0</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>19</v>
-      </c>
-      <c r="F3" t="n" s="0">
+        <v>15</v>
+      </c>
+      <c r="D3" t="n">
         <v>2.0</v>
       </c>
-      <c r="G3" t="b" s="0">
+      <c r="E3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" t="b" s="0">
+      <c r="F3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -836,21 +816,15 @@
         <v>1.0</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="D4" t="n" s="0">
-        <v>6.0</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="F4" t="n" s="0">
+        <v>16</v>
+      </c>
+      <c r="D4" t="n">
         <v>3.0</v>
       </c>
-      <c r="G4" t="b" s="0">
+      <c r="E4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" t="b" s="0">
+      <c r="F4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -862,21 +836,15 @@
         <v>6.0</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="D5" t="n" s="0">
-        <v>5.0</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="F5" t="n" s="0">
+        <v>17</v>
+      </c>
+      <c r="D5" t="n">
         <v>1.0</v>
       </c>
-      <c r="G5" t="b" s="0">
+      <c r="E5" t="b">
         <v>0</v>
       </c>
-      <c r="H5" t="b" s="0">
+      <c r="F5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -888,21 +856,15 @@
         <v>17.0</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="D6" t="n" s="0">
-        <v>8.0</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="F6" t="n" s="0">
+        <v>18</v>
+      </c>
+      <c r="D6" t="n">
         <v>1.0</v>
       </c>
-      <c r="G6" t="b" s="0">
+      <c r="E6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" t="b" s="0">
+      <c r="F6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -914,21 +876,15 @@
         <v>9.0</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="D7" t="n" s="0">
-        <v>5.0</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>23</v>
-      </c>
-      <c r="F7" t="n" s="0">
+        <v>17</v>
+      </c>
+      <c r="D7" t="n">
         <v>2.0</v>
       </c>
-      <c r="G7" t="b" s="0">
+      <c r="E7" t="b">
         <v>0</v>
       </c>
-      <c r="H7" t="b" s="0">
+      <c r="F7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -940,21 +896,15 @@
         <v>9.0</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="D8" t="n" s="0">
-        <v>16.0</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="F8" t="n" s="0">
+        <v>19</v>
+      </c>
+      <c r="D8" t="n">
         <v>1.0</v>
       </c>
-      <c r="G8" t="b" s="0">
+      <c r="E8" t="b">
         <v>1</v>
       </c>
-      <c r="H8" t="b" s="0">
+      <c r="F8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -966,21 +916,15 @@
         <v>8.0</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D9" t="n" s="0">
-        <v>2.0</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="F9" t="n" s="0">
+        <v>20</v>
+      </c>
+      <c r="D9" t="n">
         <v>3.0</v>
       </c>
-      <c r="G9" t="b" s="0">
+      <c r="E9" t="b">
         <v>1</v>
       </c>
-      <c r="H9" t="b" s="0">
+      <c r="F9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -992,21 +936,15 @@
         <v>8.0</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="D10" t="n" s="0">
-        <v>17.0</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="F10" t="n" s="0">
+        <v>21</v>
+      </c>
+      <c r="D10" t="n">
         <v>2.0</v>
       </c>
-      <c r="G10" t="b" s="0">
+      <c r="E10" t="b">
         <v>1</v>
       </c>
-      <c r="H10" t="b" s="0">
+      <c r="F10" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1020,19 +958,13 @@
       <c r="C11" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="D11" t="n" s="0">
-        <v>9.0</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="F11" t="n" s="0">
+      <c r="D11" t="n">
         <v>2.0</v>
       </c>
-      <c r="G11" t="b" s="0">
+      <c r="E11" t="b">
         <v>0</v>
       </c>
-      <c r="H11" t="b" s="0">
+      <c r="F11" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1044,21 +976,15 @@
         <v>19.0</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="D12" t="n" s="0">
-        <v>19.0</v>
-      </c>
-      <c r="E12" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="F12" t="n" s="0">
+        <v>23</v>
+      </c>
+      <c r="D12" t="n">
         <v>2.0</v>
       </c>
-      <c r="G12" t="b" s="0">
+      <c r="E12" t="b">
         <v>0</v>
       </c>
-      <c r="H12" t="b" s="0">
+      <c r="F12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1070,21 +996,15 @@
         <v>10.0</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="D13" t="n" s="0">
-        <v>15.0</v>
-      </c>
-      <c r="E13" t="s" s="0">
-        <v>34</v>
-      </c>
-      <c r="F13" t="n" s="0">
+        <v>24</v>
+      </c>
+      <c r="D13" t="n">
         <v>3.0</v>
       </c>
-      <c r="G13" t="b" s="0">
+      <c r="E13" t="b">
         <v>0</v>
       </c>
-      <c r="H13" t="b" s="0">
+      <c r="F13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1096,21 +1016,15 @@
         <v>5.0</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>35</v>
-      </c>
-      <c r="D14" t="n" s="0">
-        <v>12.0</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="F14" t="n" s="0">
+        <v>25</v>
+      </c>
+      <c r="D14" t="n">
         <v>1.0</v>
       </c>
-      <c r="G14" t="b" s="0">
+      <c r="E14" t="b">
         <v>1</v>
       </c>
-      <c r="H14" t="b" s="0">
+      <c r="F14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1122,21 +1036,15 @@
         <v>3.0</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="D15" t="n" s="0">
-        <v>17.0</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="F15" t="n" s="0">
+        <v>21</v>
+      </c>
+      <c r="D15" t="n">
         <v>3.0</v>
       </c>
-      <c r="G15" t="b" s="0">
+      <c r="E15" t="b">
         <v>0</v>
       </c>
-      <c r="H15" t="b" s="0">
+      <c r="F15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1155,13 +1063,13 @@
         <v>8</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2">
@@ -1169,13 +1077,13 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -1183,13 +1091,13 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -1197,13 +1105,13 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -1211,13 +1119,13 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
@@ -1225,13 +1133,13 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7">
@@ -1239,13 +1147,13 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8">
@@ -1253,13 +1161,13 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -1267,13 +1175,13 @@
         <v>8.0</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -1281,13 +1189,13 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11">
@@ -1295,13 +1203,13 @@
         <v>10.0</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
@@ -1309,13 +1217,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
@@ -1323,13 +1231,13 @@
         <v>12.0</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
@@ -1337,13 +1245,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -1351,13 +1259,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16">
@@ -1365,13 +1273,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17">
@@ -1379,13 +1287,13 @@
         <v>16.0</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18">
@@ -1393,13 +1301,13 @@
         <v>17.0</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19">
@@ -1407,13 +1315,13 @@
         <v>18.0</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>42</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20">
@@ -1421,13 +1329,13 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C20" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="D20" t="s" s="0">
         <v>31</v>
-      </c>
-      <c r="D20" t="s" s="0">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1445,16 +1353,16 @@
         <v>8</v>
       </c>
       <c r="B1" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="E1" t="s" s="0">
         <v>71</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>38</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>72</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>73</v>
       </c>
     </row>
     <row r="2">
@@ -1465,13 +1373,13 @@
         <v>66.0</v>
       </c>
       <c r="C2" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="E2" t="s" s="0">
         <v>74</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>75</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>76</v>
       </c>
     </row>
     <row r="3">
@@ -1482,13 +1390,13 @@
         <v>480.0</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4">
@@ -1499,13 +1407,13 @@
         <v>447.0</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -1516,13 +1424,13 @@
         <v>256.0</v>
       </c>
       <c r="C5" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>80</v>
+      </c>
+      <c r="E5" t="s" s="0">
         <v>81</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>82</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>83</v>
       </c>
     </row>
     <row r="6">
@@ -1533,13 +1441,13 @@
         <v>313.0</v>
       </c>
       <c r="C6" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E6" t="s" s="0">
         <v>84</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>85</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>86</v>
       </c>
     </row>
     <row r="7">
@@ -1550,13 +1458,13 @@
         <v>421.0</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8">
@@ -1567,13 +1475,13 @@
         <v>323.0</v>
       </c>
       <c r="C8" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="E8" t="s" s="0">
         <v>88</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>89</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>90</v>
       </c>
     </row>
     <row r="9">
@@ -1584,13 +1492,13 @@
         <v>398.0</v>
       </c>
       <c r="C9" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="E9" t="s" s="0">
         <v>91</v>
-      </c>
-      <c r="D9" t="s" s="0">
-        <v>92</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>93</v>
       </c>
     </row>
     <row r="10">
@@ -1601,13 +1509,13 @@
         <v>488.0</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11">
@@ -1618,13 +1526,13 @@
         <v>125.0</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>45</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1634,24 +1542,21 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>99</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2">
@@ -1659,16 +1564,13 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>57</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -1676,16 +1578,13 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>28</v>
+        <v>101</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>105</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
@@ -1693,16 +1592,13 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>19</v>
+        <v>104</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>108</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>60</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5">
@@ -1710,16 +1606,13 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>111</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6">
@@ -1727,16 +1620,13 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>23</v>
+        <v>110</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>57</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -1744,16 +1634,13 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>21</v>
+        <v>112</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>115</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8">
@@ -1761,16 +1648,13 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="E8" t="s" s="0">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9">
@@ -1778,16 +1662,13 @@
         <v>8.0</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>25</v>
+        <v>118</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>122</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
@@ -1795,16 +1676,13 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>124</v>
-      </c>
-      <c r="E10" t="s" s="0">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11">
@@ -1812,16 +1690,13 @@
         <v>10.0</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>128</v>
-      </c>
-      <c r="E11" t="s" s="0">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12">
@@ -1829,16 +1704,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>131</v>
-      </c>
-      <c r="E12" t="s" s="0">
-        <v>33</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13">
@@ -1846,16 +1718,13 @@
         <v>12.0</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>36</v>
+        <v>129</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>133</v>
-      </c>
-      <c r="E13" t="s" s="0">
-        <v>64</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
@@ -1863,16 +1732,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>103</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>57</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -1880,16 +1746,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>138</v>
-      </c>
-      <c r="E15" t="s" s="0">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="16">
@@ -1897,16 +1760,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>34</v>
+        <v>136</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>141</v>
-      </c>
-      <c r="E16" t="s" s="0">
-        <v>48</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17">
@@ -1914,16 +1774,13 @@
         <v>16.0</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>27</v>
+        <v>139</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>143</v>
-      </c>
-      <c r="E17" t="s" s="0">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18">
@@ -1931,16 +1788,13 @@
         <v>17.0</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>29</v>
+        <v>142</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>146</v>
-      </c>
-      <c r="E18" t="s" s="0">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19">
@@ -1948,16 +1802,13 @@
         <v>18.0</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>150</v>
-      </c>
-      <c r="E19" t="s" s="0">
-        <v>151</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20">
@@ -1965,16 +1816,13 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>153</v>
-      </c>
-      <c r="E20" t="s" s="0">
-        <v>154</v>
+        <v>149</v>
       </c>
     </row>
     <row r="21">
@@ -1982,16 +1830,13 @@
         <v>20.0</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>157</v>
-      </c>
-      <c r="E21" t="s" s="0">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
subject color frontend error handling
</commit_message>
<xml_diff>
--- a/leo-planer/src/files/excelFiles/export/test1.xlsx
+++ b/leo-planer/src/files/excelFiles/export/test1.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="154">
   <si>
     <t>CSI Id</t>
   </si>
@@ -49,6 +49,9 @@
   </si>
   <si>
     <t>Teacher Ids</t>
+  </si>
+  <si>
+    <t>School class ID</t>
   </si>
   <si>
     <t>Weekly Hours</t>
@@ -519,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -591,7 +594,7 @@
         <v>4.0</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="7">
@@ -607,7 +610,7 @@
         <v>6.0</v>
       </c>
       <c r="B8" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="9">
@@ -615,7 +618,7 @@
         <v>7.0</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="10">
@@ -623,7 +626,7 @@
         <v>8.0</v>
       </c>
       <c r="B10" t="n" s="0">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="11">
@@ -639,7 +642,7 @@
         <v>10.0</v>
       </c>
       <c r="B12" t="n" s="0">
-        <v>7.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="13">
@@ -647,7 +650,7 @@
         <v>11.0</v>
       </c>
       <c r="B13" t="n" s="0">
-        <v>8.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="14">
@@ -663,7 +666,7 @@
         <v>13.0</v>
       </c>
       <c r="B15" t="n" s="0">
-        <v>9.0</v>
+        <v>8.0</v>
       </c>
     </row>
     <row r="16">
@@ -679,7 +682,7 @@
         <v>15.0</v>
       </c>
       <c r="B17" t="n" s="0">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="18">
@@ -687,7 +690,7 @@
         <v>16.0</v>
       </c>
       <c r="B18" t="n" s="0">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="19">
@@ -695,7 +698,7 @@
         <v>17.0</v>
       </c>
       <c r="B19" t="n" s="0">
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="20">
@@ -703,7 +706,7 @@
         <v>18.0</v>
       </c>
       <c r="B20" t="n" s="0">
-        <v>12.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="21">
@@ -719,7 +722,7 @@
         <v>20.0</v>
       </c>
       <c r="B22" t="n" s="0">
-        <v>13.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="23">
@@ -727,7 +730,7 @@
         <v>21.0</v>
       </c>
       <c r="B23" t="n" s="0">
-        <v>14.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="24">
@@ -735,6 +738,14 @@
         <v>22.0</v>
       </c>
       <c r="B24" t="n" s="0">
+        <v>14.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n" s="0">
+        <v>23.0</v>
+      </c>
+      <c r="B25" t="n" s="0">
         <v>14.0</v>
       </c>
     </row>
@@ -745,7 +756,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -767,6 +778,9 @@
       <c r="F1" t="s" s="0">
         <v>13</v>
       </c>
+      <c r="G1" t="s" s="0">
+        <v>14</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
@@ -776,15 +790,18 @@
         <v>8.0</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E2" t="n">
         <v>2.0</v>
       </c>
-      <c r="E2" t="b">
+      <c r="F2" t="b">
         <v>1</v>
       </c>
-      <c r="F2" t="b">
+      <c r="G2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -796,15 +813,18 @@
         <v>12.0</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E3" t="n">
         <v>2.0</v>
       </c>
-      <c r="E3" t="b">
+      <c r="F3" t="b">
         <v>1</v>
       </c>
-      <c r="F3" t="b">
+      <c r="G3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -816,15 +836,18 @@
         <v>1.0</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E4" t="n">
         <v>3.0</v>
       </c>
-      <c r="E4" t="b">
+      <c r="F4" t="b">
         <v>1</v>
       </c>
-      <c r="F4" t="b">
+      <c r="G4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -836,15 +859,18 @@
         <v>6.0</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" t="n">
         <v>1.0</v>
       </c>
-      <c r="E5" t="b">
+      <c r="E5" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F5" t="b">
         <v>0</v>
       </c>
-      <c r="F5" t="b">
+      <c r="G5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -856,15 +882,18 @@
         <v>17.0</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" t="n">
         <v>1.0</v>
       </c>
-      <c r="E6" t="b">
+      <c r="E6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F6" t="b">
         <v>1</v>
       </c>
-      <c r="F6" t="b">
+      <c r="G6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -876,15 +905,18 @@
         <v>9.0</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D7" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E7" t="n">
         <v>2.0</v>
       </c>
-      <c r="E7" t="b">
+      <c r="F7" t="b">
         <v>0</v>
       </c>
-      <c r="F7" t="b">
+      <c r="G7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -896,15 +928,18 @@
         <v>9.0</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D8" t="n">
         <v>1.0</v>
       </c>
-      <c r="E8" t="b">
+      <c r="E8" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F8" t="b">
         <v>1</v>
       </c>
-      <c r="F8" t="b">
+      <c r="G8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -916,15 +951,18 @@
         <v>8.0</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E9" t="n">
         <v>3.0</v>
       </c>
-      <c r="E9" t="b">
+      <c r="F9" t="b">
         <v>1</v>
       </c>
-      <c r="F9" t="b">
+      <c r="G9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -936,15 +974,18 @@
         <v>8.0</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E10" t="n">
         <v>2.0</v>
       </c>
-      <c r="E10" t="b">
+      <c r="F10" t="b">
         <v>1</v>
       </c>
-      <c r="F10" t="b">
+      <c r="G10" t="b">
         <v>1</v>
       </c>
     </row>
@@ -956,15 +997,18 @@
         <v>6.0</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D11" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E11" t="n">
         <v>2.0</v>
       </c>
-      <c r="E11" t="b">
+      <c r="F11" t="b">
         <v>0</v>
       </c>
-      <c r="F11" t="b">
+      <c r="G11" t="b">
         <v>1</v>
       </c>
     </row>
@@ -976,15 +1020,18 @@
         <v>19.0</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D12" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E12" t="n">
         <v>2.0</v>
       </c>
-      <c r="E12" t="b">
+      <c r="F12" t="b">
         <v>0</v>
       </c>
-      <c r="F12" t="b">
+      <c r="G12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -996,15 +1043,18 @@
         <v>10.0</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E13" t="n">
         <v>3.0</v>
       </c>
-      <c r="E13" t="b">
+      <c r="F13" t="b">
         <v>0</v>
       </c>
-      <c r="F13" t="b">
+      <c r="G13" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1016,15 +1066,18 @@
         <v>5.0</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D14" t="n">
         <v>1.0</v>
       </c>
-      <c r="E14" t="b">
+      <c r="E14" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F14" t="b">
         <v>1</v>
       </c>
-      <c r="F14" t="b">
+      <c r="G14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1036,15 +1089,18 @@
         <v>3.0</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D15" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E15" t="n">
         <v>3.0</v>
       </c>
-      <c r="E15" t="b">
+      <c r="F15" t="b">
         <v>0</v>
       </c>
-      <c r="F15" t="b">
+      <c r="G15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1063,13 +1119,13 @@
         <v>8</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2">
@@ -1077,13 +1133,13 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -1091,13 +1147,13 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -1105,13 +1161,13 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -1119,13 +1175,13 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -1133,13 +1189,13 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
@@ -1147,13 +1203,13 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
@@ -1161,13 +1217,13 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
@@ -1175,13 +1231,13 @@
         <v>8.0</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
@@ -1189,13 +1245,13 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11">
@@ -1203,13 +1259,13 @@
         <v>10.0</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -1217,13 +1273,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13">
@@ -1231,13 +1287,13 @@
         <v>12.0</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
@@ -1245,13 +1301,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
@@ -1259,13 +1315,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16">
@@ -1273,13 +1329,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
@@ -1287,13 +1343,13 @@
         <v>16.0</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18">
@@ -1301,13 +1357,13 @@
         <v>17.0</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19">
@@ -1315,13 +1371,13 @@
         <v>18.0</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20">
@@ -1329,13 +1385,13 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1353,16 +1409,16 @@
         <v>8</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2">
@@ -1373,13 +1429,13 @@
         <v>66.0</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
@@ -1390,13 +1446,13 @@
         <v>480.0</v>
       </c>
       <c r="C3" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="E3" t="s" s="0">
         <v>75</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>76</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>74</v>
       </c>
     </row>
     <row r="4">
@@ -1407,13 +1463,13 @@
         <v>447.0</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
@@ -1424,13 +1480,13 @@
         <v>256.0</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6">
@@ -1441,13 +1497,13 @@
         <v>313.0</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7">
@@ -1458,13 +1514,13 @@
         <v>421.0</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8">
@@ -1475,13 +1531,13 @@
         <v>323.0</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9">
@@ -1492,13 +1548,13 @@
         <v>398.0</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10">
@@ -1509,13 +1565,13 @@
         <v>488.0</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11">
@@ -1526,13 +1582,13 @@
         <v>125.0</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1547,16 +1603,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2">
@@ -1564,13 +1620,13 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -1578,13 +1634,13 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4">
@@ -1592,13 +1648,13 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5">
@@ -1606,13 +1662,13 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
@@ -1620,13 +1676,13 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -1634,13 +1690,13 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8">
@@ -1648,13 +1704,13 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9">
@@ -1662,13 +1718,13 @@
         <v>8.0</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -1676,13 +1732,13 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11">
@@ -1690,13 +1746,13 @@
         <v>10.0</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12">
@@ -1704,13 +1760,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13">
@@ -1718,13 +1774,13 @@
         <v>12.0</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -1732,13 +1788,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -1746,13 +1802,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16">
@@ -1760,13 +1816,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="17">
@@ -1774,13 +1830,13 @@
         <v>16.0</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18">
@@ -1788,13 +1844,13 @@
         <v>17.0</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19">
@@ -1802,13 +1858,13 @@
         <v>18.0</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20">
@@ -1816,13 +1872,13 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21">
@@ -1830,13 +1886,13 @@
         <v>20.0</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>